<commit_message>
Templates: red * on required columns; the import reads 'Title *' as Title
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import-templates/Bibliography import template.xlsx
+++ b/import-templates/Bibliography import template.xlsx
@@ -55,7 +55,23 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Type</t>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve">Type</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <color rgb="FFFF0000"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve"> *</t>
+          </r>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
@@ -70,12 +86,44 @@
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Names</t>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve">Names</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <color rgb="FFFF0000"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve"> *</t>
+          </r>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">Title</t>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve">Title</t>
+          </r>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="11"/>
+              <color rgb="FFFF0000"/>
+              <rFont val="Calibri"/>
+            </rPr>
+            <t xml:space="preserve"> *</t>
+          </r>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
@@ -866,7 +914,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Column names must be spelled exactly as in row 1. Keep row 1 as the headers. Save/download as .xlsx. The Keywords tab pairs each keyword with its translation. This tab is ignored by the import.</t>
+          <t xml:space="preserve">A red * marks a required column. Column names must be spelled exactly as in row 1 (the * can stay or go). Keep row 1 as the headers. Save/download as .xlsx. The Keywords tab pairs each keyword with its translation. This tab is ignored by the import.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Templates: unambiguous Copyright status and Type lists; DOI alone gives no link
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import-templates/Bibliography import template.xlsx
+++ b/import-templates/Bibliography import template.xlsx
@@ -559,7 +559,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Book / Book chapter / Journal article / Other article / Report / Thesis / From website. Anything else becomes Other.</t>
+          <t xml:space="preserve">One of: Book ; Book chapter ; Journal article ; Other article ; Report ; Thesis ; From website. Anything else becomes Other.</t>
         </is>
       </c>
     </row>
@@ -804,7 +804,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Link to the source. Entries with a URL show as links, without one as citations.</t>
+          <t xml:space="preserve">Link to the source. Entries with a URL show on the website as citation + link; without one, as citation only. A DOI alone does not make a link, so put the link here too.</t>
         </is>
       </c>
     </row>
@@ -867,7 +867,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copyrighted / Copyrighted / verify / Public domain / Open access / verify licence / Web content / verify terms</t>
+          <t xml:space="preserve">Exactly one of these five (copy one whole): "Copyrighted" ; "Copyrighted / verify" ; "Public domain" ; "Open access / verify licence" ; "Web content / verify terms". Anything else is left empty.</t>
         </is>
       </c>
     </row>

</xml_diff>